<commit_message>
// SOAP  soil WB
</commit_message>
<xml_diff>
--- a/auxfiles/GSSHApedotransfer.xlsx
+++ b/auxfiles/GSSHApedotransfer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\prgc\lisemgit\openlisem\auxfiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE2F88C-1CCB-414C-8123-D1CE6FBDB79F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A77C74-1346-46C3-AAF0-56854B3C9902}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{EE7E3014-B43F-4E75-BCA9-657834F4F7BD}"/>
   </bookViews>
@@ -541,410 +541,6 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="nl-NL"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:noFill/>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:trendline>
-            <c:spPr>
-              <a:ln w="19050" cap="rnd">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-                <a:prstDash val="sysDot"/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:trendlineType val="log"/>
-            <c:dispRSqr val="1"/>
-            <c:dispEq val="1"/>
-            <c:trendlineLbl>
-              <c:layout>
-                <c:manualLayout>
-                  <c:x val="7.7099737532808396E-2"/>
-                  <c:y val="0.42082421988918062"/>
-                </c:manualLayout>
-              </c:layout>
-              <c:numFmt formatCode="General" sourceLinked="0"/>
-              <c:spPr>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="65000"/>
-                          <a:lumOff val="35000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:latin typeface="+mn-lt"/>
-                      <a:ea typeface="+mn-ea"/>
-                      <a:cs typeface="+mn-cs"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="nl-NL"/>
-                </a:p>
-              </c:txPr>
-            </c:trendlineLbl>
-          </c:trendline>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Sheet1!$S$8:$S$18</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
-                <c:pt idx="0">
-                  <c:v>235.6</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>59.800000000000004</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>21.8</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>13.200000000000001</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>6.8000000000000007</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.6</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$Z$8:$Z$18</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
-                <c:pt idx="0">
-                  <c:v>0.69399999999999995</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.55300000000000005</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.378</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.252</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.23400000000000001</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.31900000000000001</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.24199999999999999</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.17699999999999999</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.223</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.15</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.16500000000000001</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-EEAB-4542-B7F9-EAD1D340D214}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="1958512127"/>
-        <c:axId val="1958513087"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="1958512127"/>
-        <c:scaling>
-          <c:logBase val="10"/>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1958513087"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="1958513087"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1958512127"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="nl-NL"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
       <c:tx>
         <c:rich>
           <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
@@ -965,818 +561,11 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="nl-NL"/>
-              <a:t>ln(bub) = ln(ks)</a:t>
+              <a:t>ln(lambda)=f(ln(ks))</a:t>
             </a:r>
           </a:p>
         </c:rich>
       </c:tx>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="nl-NL"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:noFill/>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:trendline>
-            <c:spPr>
-              <a:ln w="19050" cap="rnd">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-                <a:prstDash val="sysDot"/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:trendlineType val="linear"/>
-            <c:dispRSqr val="1"/>
-            <c:dispEq val="1"/>
-            <c:trendlineLbl>
-              <c:layout>
-                <c:manualLayout>
-                  <c:x val="-9.5097331583552061E-2"/>
-                  <c:y val="0.11358267716535433"/>
-                </c:manualLayout>
-              </c:layout>
-              <c:numFmt formatCode="General" sourceLinked="0"/>
-              <c:spPr>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="65000"/>
-                          <a:lumOff val="35000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:latin typeface="+mn-lt"/>
-                      <a:ea typeface="+mn-ea"/>
-                      <a:cs typeface="+mn-cs"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="nl-NL"/>
-                </a:p>
-              </c:txPr>
-            </c:trendlineLbl>
-          </c:trendline>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Sheet1!$AA$8:$AA$18</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
-                <c:pt idx="0">
-                  <c:v>5.4621354517774314</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>4.0910056609565864</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>3.0819099697950434</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2.5802168295923251</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.9169226121820611</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1.0986122886681098</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.69314718055994529</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.69314718055994529</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.18232155679395459</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>-0.51082562376599072</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$AC$8:$AC$18</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
-                <c:pt idx="0">
-                  <c:v>1.9823798288367047</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>2.1621729392773008</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2.6851226964585053</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2.411439497906128</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>3.0344721018699214</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>3.3350575791576103</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>3.2538567937634464</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>3.4830845411343394</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>3.3731407838796299</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>3.5319332036512097</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>3.6189933266497696</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C89F-4724-8285-2B34186920FD}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="1774120032"/>
-        <c:axId val="1774120512"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="1774120032"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1774120512"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="1774120512"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1774120032"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="nl-NL"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="nl-NL"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:noFill/>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:trendline>
-            <c:spPr>
-              <a:ln w="19050" cap="rnd">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-                <a:prstDash val="sysDot"/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:trendlineType val="log"/>
-            <c:dispRSqr val="1"/>
-            <c:dispEq val="1"/>
-            <c:trendlineLbl>
-              <c:layout>
-                <c:manualLayout>
-                  <c:x val="-0.438247375328084"/>
-                  <c:y val="-0.17977653834937299"/>
-                </c:manualLayout>
-              </c:layout>
-              <c:numFmt formatCode="General" sourceLinked="0"/>
-              <c:spPr>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="65000"/>
-                          <a:lumOff val="35000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:latin typeface="+mn-lt"/>
-                      <a:ea typeface="+mn-ea"/>
-                      <a:cs typeface="+mn-cs"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="nl-NL"/>
-                </a:p>
-              </c:txPr>
-            </c:trendlineLbl>
-          </c:trendline>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Sheet1!$P$8:$P$18</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
-                <c:pt idx="0">
-                  <c:v>23.56</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>5.98</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2.1800000000000002</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.32</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.68</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.3</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.2</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.2</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.12</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.06</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$Q$8:$Q$18</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
-                <c:pt idx="0">
-                  <c:v>4.95</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>6.13</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>11.01</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>8.89</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>16.68</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>21.85</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>20.88</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>27.3</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>23.9</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>29.22</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>31.63</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-6609-43B2-B495-282969FE61C8}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="825487487"/>
-        <c:axId val="825484127"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="825487487"/>
-        <c:scaling>
-          <c:logBase val="10"/>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="825484127"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="825484127"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="825487487"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="nl-NL"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2165,410 +954,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="nl-NL"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:noFill/>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:trendline>
-            <c:spPr>
-              <a:ln w="19050" cap="rnd">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-                <a:prstDash val="sysDot"/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:trendlineType val="log"/>
-            <c:dispRSqr val="1"/>
-            <c:dispEq val="1"/>
-            <c:trendlineLbl>
-              <c:layout>
-                <c:manualLayout>
-                  <c:x val="-9.7686570428696412E-2"/>
-                  <c:y val="-0.41588764946048412"/>
-                </c:manualLayout>
-              </c:layout>
-              <c:numFmt formatCode="General" sourceLinked="0"/>
-              <c:spPr>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="65000"/>
-                          <a:lumOff val="35000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:latin typeface="+mn-lt"/>
-                      <a:ea typeface="+mn-ea"/>
-                      <a:cs typeface="+mn-cs"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="nl-NL"/>
-                </a:p>
-              </c:txPr>
-            </c:trendlineLbl>
-          </c:trendline>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Sheet1!$S$8:$S$18</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
-                <c:pt idx="0">
-                  <c:v>235.6</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>59.800000000000004</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>21.8</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>13.200000000000001</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>6.8000000000000007</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.6</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$T$8:$T$18</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="11"/>
-                <c:pt idx="0">
-                  <c:v>4.95</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>6.13</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>11.01</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>8.89</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>16.68</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>21.85</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>20.88</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>27.3</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>23.9</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>29.22</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>31.63</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-EDF7-4873-8BFC-B1ACBCF40D78}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="349207504"/>
-        <c:axId val="349209424"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="349207504"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="349209424"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="349209424"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="349207504"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="nl-NL"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -3129,7 +1515,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -3565,7 +1951,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -4001,7 +2387,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -4439,7 +2825,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -4792,47 +3178,901 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="nl-NL"/>
+              <a:t>ln(bub) = ln(ks)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="nl-NL"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-9.5097331583552061E-2"/>
+                  <c:y val="0.11358267716535433"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="nl-NL"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$AA$8:$AA$18</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>5.4621354517774314</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.0910056609565864</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.0819099697950434</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.5802168295923251</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.9169226121820611</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.0986122886681098</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.69314718055994529</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.69314718055994529</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.18232155679395459</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-0.51082562376599072</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$AC$8:$AC$18</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>1.9823798288367047</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.1621729392773008</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.6851226964585053</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.411439497906128</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3.0344721018699214</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3.3350575791576103</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>3.2538567937634464</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.4830845411343394</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>3.3731407838796299</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>3.5319332036512097</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>3.6189933266497696</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C89F-4724-8285-2B34186920FD}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1774120032"/>
+        <c:axId val="1774120512"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1774120032"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="nl-NL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1774120512"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1774120512"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="nl-NL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1774120032"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="nl-NL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
 </file>
 
-<file path=xl/charts/colors10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="nl-NL"/>
+              <a:t>lambda=f(ln(ks))</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="nl-NL"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="nl-NL"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="exp"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="nl-NL"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$X$8:$X$18</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>5.4621354517774314</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.0910056609565864</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.0819099697950434</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.5802168295923251</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.9169226121820611</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.0986122886681098</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.69314718055994529</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.69314718055994529</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.18232155679395459</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-0.51082562376599072</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$Z$8:$Z$18</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>0.69399999999999995</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.55300000000000005</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.378</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.252</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.23400000000000001</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.31900000000000001</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.24199999999999999</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.17699999999999999</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.223</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.15</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.16500000000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F242-407F-936E-F043C3330488}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="167585584"/>
+        <c:axId val="167440672"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="167585584"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="nl-NL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="167440672"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="167440672"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="nl-NL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="167585584"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="nl-NL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -5152,46 +4392,6 @@
 </cs:colorStyle>
 </file>
 
-<file path=xl/charts/colors9.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -5708,7 +4908,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -6224,7 +5424,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -6740,7 +5940,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -7256,7 +6456,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -7772,7 +6972,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -8288,7 +7488,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style7.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -8804,1039 +8004,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style7.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/charts/style8.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/charts/style9.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -10480,88 +8648,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>32</xdr:col>
-      <xdr:colOff>371475</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>4762</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>40</xdr:col>
-      <xdr:colOff>66675</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>233362</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{578237E3-32CB-D0FF-F7EC-7DF110ED4D33}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>31</xdr:col>
-      <xdr:colOff>353376</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>60007</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>42</xdr:col>
-      <xdr:colOff>15239</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>118110</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="6" name="Chart 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{210AF32C-16DE-86ED-FECD-E149BFD8B496}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>26</xdr:col>
       <xdr:colOff>23812</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>128587</xdr:rowOff>
+      <xdr:rowOff>128586</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>33</xdr:col>
       <xdr:colOff>328612</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>204787</xdr:rowOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>342899</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -10580,43 +8676,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>74295</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>50482</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>35</xdr:col>
-      <xdr:colOff>379095</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>75247</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Chart 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CDCFEE56-6675-0C5A-3777-C657F53B1E03}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10652,7 +8712,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10660,16 +8720,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>50483</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>107631</xdr:rowOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>153351</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>355283</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>176211</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>39051</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -10688,7 +8748,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10724,7 +8784,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10760,7 +8820,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10796,7 +8856,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10804,16 +8864,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>137160</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>68580</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>441960</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>68580</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -10832,7 +8892,43 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>259080</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>563880</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="9" name="Chart 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00E765DF-F950-EBE9-39A3-10C853A2D052}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -12199,6 +10295,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="c2fb78ee-7f80-47d5-98b2-7e891369b7bb" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B3BEC45979C5C049A19F02E744A428FF" ma:contentTypeVersion="14" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="f5996e32557378a90493e5f03249e0f6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="c2fb78ee-7f80-47d5-98b2-7e891369b7bb" xmlns:ns4="8e80448a-be4d-46ae-83bb-e2adae7741fa" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0d0d7db69a812adcd006be6af9aa5ff0" ns3:_="" ns4:_="">
     <xsd:import namespace="c2fb78ee-7f80-47d5-98b2-7e891369b7bb"/>
@@ -12427,38 +10540,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="c2fb78ee-7f80-47d5-98b2-7e891369b7bb" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{212E6E55-4940-49C5-A955-F25080F8975C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{546FAC25-7A53-4BE4-87D4-6463C2D97D48}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c2fb78ee-7f80-47d5-98b2-7e891369b7bb"/>
-    <ds:schemaRef ds:uri="8e80448a-be4d-46ae-83bb-e2adae7741fa"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -12481,9 +10566,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{546FAC25-7A53-4BE4-87D4-6463C2D97D48}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{212E6E55-4940-49C5-A955-F25080F8975C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c2fb78ee-7f80-47d5-98b2-7e891369b7bb"/>
+    <ds:schemaRef ds:uri="8e80448a-be4d-46ae-83bb-e2adae7741fa"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
//works reserve in QVector does not work
</commit_message>
<xml_diff>
--- a/auxfiles/GSSHApedotransfer.xlsx
+++ b/auxfiles/GSSHApedotransfer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\prgc\lisemgit\openlisem\auxfiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A77C74-1346-46C3-AAF0-56854B3C9902}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B3459DB-E169-468E-A79E-D7714708172C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{EE7E3014-B43F-4E75-BCA9-657834F4F7BD}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="50">
   <si>
     <t>Sand</t>
   </si>
@@ -331,6 +331,9 @@
   <si>
     <t>ln(bub)</t>
   </si>
+  <si>
+    <t>ln(thetar)</t>
+  </si>
 </sst>
 </file>
 
@@ -478,7 +481,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -508,6 +511,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4072,6 +4076,448 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="nl-NL"/>
+              <a:t>thetar</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="nl-NL"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="power"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="exp"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-8.8075240594925643E-3"/>
+                  <c:y val="-0.41454651501895595"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="nl-NL"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$H$8:$H$18</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>5.4621354517774314</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4.0910056609565864</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.0819099697950434</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.5802168295923251</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.9169226121820611</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.0986122886681098</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.69314718055994529</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.69314718055994529</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.18232155679395459</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-0.51082562376599072</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$M$8:$M$18</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>0.02</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.5000000000000003E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4.1000000000000002E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2.7E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.4999999999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6.8000000000000005E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7.4999999999999997E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.04</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.109</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>5.6000000000000001E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.09</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-14A3-4776-8BEC-D602FD9243F2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="2009214831"/>
+        <c:axId val="2009216271"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="2009214831"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="nl-NL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2009216271"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="2009216271"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="nl-NL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2009214831"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="nl-NL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -4392,6 +4838,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors9.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -8005,6 +8491,522 @@
 </file>
 
 <file path=xl/charts/style8.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style9.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -8720,16 +9722,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>50483</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>153351</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>195263</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>298131</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>355283</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>39051</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>500063</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>951</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8792,16 +9794,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>233841</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>115253</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>81441</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>122873</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>538641</xdr:colOff>
-      <xdr:row>56</xdr:row>
-      <xdr:rowOff>16193</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>386241</xdr:colOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>23813</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8929,6 +9931,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>45720</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>350520</xdr:colOff>
+      <xdr:row>61</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B0E7327E-F6E3-FEBF-543F-08766C4E78DC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -9234,7 +10272,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AC7A993-96B8-4AA6-8EF4-C236C394CA84}">
-  <dimension ref="F1:AC18"/>
+  <dimension ref="F1:AC54"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="8" max="8" width="12.109375" bestFit="1" customWidth="1"/>
@@ -9353,6 +10391,9 @@
       <c r="Q6" s="2" t="s">
         <v>25</v>
       </c>
+      <c r="R6" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="S6" s="2" t="s">
         <v>35</v>
       </c>
@@ -9438,6 +10479,10 @@
       <c r="Q8" s="2">
         <v>4.95</v>
       </c>
+      <c r="R8">
+        <f>LN(M8)</f>
+        <v>-3.912023005428146</v>
+      </c>
       <c r="S8">
         <f>P8*10</f>
         <v>235.6</v>
@@ -9518,28 +10563,32 @@
       <c r="Q9" s="2">
         <v>6.13</v>
       </c>
+      <c r="R9">
+        <f t="shared" ref="R9:R18" si="4">LN(M9)</f>
+        <v>-3.3524072174927233</v>
+      </c>
       <c r="S9">
-        <f t="shared" ref="S9:S18" si="4">P9*10</f>
+        <f t="shared" ref="S9:S18" si="5">P9*10</f>
         <v>59.800000000000004</v>
       </c>
       <c r="T9">
-        <f t="shared" ref="T9:T18" si="5">Q9</f>
+        <f t="shared" ref="T9:T18" si="6">Q9</f>
         <v>6.13</v>
       </c>
       <c r="V9">
-        <f t="shared" ref="V9:V18" si="6">LOG(S9)</f>
+        <f t="shared" ref="V9:V18" si="7">LOG(S9)</f>
         <v>1.7767011839884108</v>
       </c>
       <c r="W9">
-        <f t="shared" ref="W9:W18" si="7">LOG(T9)</f>
+        <f t="shared" ref="W9:W18" si="8">LOG(T9)</f>
         <v>0.78746047451841505</v>
       </c>
       <c r="X9">
-        <f t="shared" ref="X9:X18" si="8">LN(S9)</f>
+        <f t="shared" ref="X9:X18" si="9">LN(S9)</f>
         <v>4.0910056609565864</v>
       </c>
       <c r="Y9">
-        <f t="shared" ref="Y9:Y18" si="9">LN(T9)</f>
+        <f t="shared" ref="Y9:Y18" si="10">LN(T9)</f>
         <v>1.81319474994812</v>
       </c>
       <c r="Z9">
@@ -9551,11 +10600,11 @@
         <v>4.0910056609565864</v>
       </c>
       <c r="AB9">
-        <f t="shared" ref="AB9:AB18" si="10">LN(Z9)</f>
+        <f t="shared" ref="AB9:AB18" si="11">LN(Z9)</f>
         <v>-0.5923972774598022</v>
       </c>
       <c r="AC9">
-        <f t="shared" ref="AC9:AC18" si="11">LN(N9)</f>
+        <f t="shared" ref="AC9:AC18" si="12">LN(N9)</f>
         <v>2.1621729392773008</v>
       </c>
     </row>
@@ -9598,28 +10647,32 @@
       <c r="Q10" s="2">
         <v>11.01</v>
       </c>
+      <c r="R10">
+        <f t="shared" si="4"/>
+        <v>-3.1941832122778293</v>
+      </c>
       <c r="S10">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>21.8</v>
       </c>
       <c r="T10">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>11.01</v>
       </c>
       <c r="V10">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1.3384564936046048</v>
       </c>
       <c r="W10">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.0417873189717517</v>
       </c>
       <c r="X10">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>3.0819099697950434</v>
       </c>
       <c r="Y10">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>2.3988039507345884</v>
       </c>
       <c r="Z10">
@@ -9631,11 +10684,11 @@
         <v>3.0819099697950434</v>
       </c>
       <c r="AB10">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-0.97286108336254939</v>
       </c>
       <c r="AC10">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>2.6851226964585053</v>
       </c>
     </row>
@@ -9678,28 +10731,32 @@
       <c r="Q11" s="2">
         <v>8.89</v>
       </c>
+      <c r="R11">
+        <f t="shared" si="4"/>
+        <v>-3.6119184129778081</v>
+      </c>
       <c r="S11">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>13.200000000000001</v>
       </c>
       <c r="T11">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>8.89</v>
       </c>
       <c r="V11">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>1.1205739312058498</v>
       </c>
       <c r="W11">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.94890176097021373</v>
       </c>
       <c r="X11">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>2.5802168295923251</v>
       </c>
       <c r="Y11">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>2.1849270495258133</v>
       </c>
       <c r="Z11">
@@ -9711,11 +10768,11 @@
         <v>2.5802168295923251</v>
       </c>
       <c r="AB11">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-1.3783261914707137</v>
       </c>
       <c r="AC11">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>2.411439497906128</v>
       </c>
     </row>
@@ -9758,28 +10815,32 @@
       <c r="Q12" s="2">
         <v>16.68</v>
       </c>
+      <c r="R12">
+        <f t="shared" si="4"/>
+        <v>-4.1997050778799272</v>
+      </c>
       <c r="S12">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>6.8000000000000007</v>
       </c>
       <c r="T12">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>16.68</v>
       </c>
       <c r="V12">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.83250891270623639</v>
       </c>
       <c r="W12">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.2221960463017199</v>
       </c>
       <c r="X12">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1.9169226121820611</v>
       </c>
       <c r="Y12">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>2.8142103969306005</v>
       </c>
       <c r="Z12">
@@ -9791,11 +10852,11 @@
         <v>1.9169226121820611</v>
       </c>
       <c r="AB12">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-1.4524341636244356</v>
       </c>
       <c r="AC12">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3.0344721018699214</v>
       </c>
     </row>
@@ -9838,28 +10899,32 @@
       <c r="Q13" s="2">
         <v>21.85</v>
       </c>
+      <c r="R13">
+        <f t="shared" si="4"/>
+        <v>-2.6882475738060303</v>
+      </c>
       <c r="S13">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>3</v>
       </c>
       <c r="T13">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>21.85</v>
       </c>
       <c r="V13">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.47712125471966244</v>
       </c>
       <c r="W13">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.3394514413064407</v>
       </c>
       <c r="X13">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1.0986122886681098</v>
       </c>
       <c r="Y13">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>3.0842009215415991</v>
       </c>
       <c r="Z13">
@@ -9871,11 +10936,11 @@
         <v>1.0986122886681098</v>
       </c>
       <c r="AB13">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-1.1425641761972924</v>
       </c>
       <c r="AC13">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3.3350575791576103</v>
       </c>
     </row>
@@ -9918,28 +10983,32 @@
       <c r="Q14" s="2">
         <v>20.88</v>
       </c>
+      <c r="R14">
+        <f t="shared" si="4"/>
+        <v>-2.5902671654458267</v>
+      </c>
       <c r="S14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="T14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>20.88</v>
       </c>
       <c r="V14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.3010299956639812</v>
       </c>
       <c r="W14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.3197304943302246</v>
       </c>
       <c r="X14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.69314718055994529</v>
       </c>
       <c r="Y14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>3.0387917630144381</v>
       </c>
       <c r="Z14">
@@ -9951,11 +11020,11 @@
         <v>0.69314718055994529</v>
       </c>
       <c r="AB14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-1.4188175528254507</v>
       </c>
       <c r="AC14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3.2538567937634464</v>
       </c>
     </row>
@@ -9998,28 +11067,32 @@
       <c r="Q15" s="2">
         <v>27.3</v>
       </c>
+      <c r="R15">
+        <f t="shared" si="4"/>
+        <v>-3.2188758248682006</v>
+      </c>
       <c r="S15">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>2</v>
       </c>
       <c r="T15">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>27.3</v>
       </c>
       <c r="V15">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.3010299956639812</v>
       </c>
       <c r="W15">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.436162647040756</v>
       </c>
       <c r="X15">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.69314718055994529</v>
       </c>
       <c r="Y15">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>3.3068867021909143</v>
       </c>
       <c r="Z15">
@@ -10031,11 +11104,11 @@
         <v>0.69314718055994529</v>
       </c>
       <c r="AB15">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-1.731605546408308</v>
       </c>
       <c r="AC15">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3.4830845411343394</v>
       </c>
     </row>
@@ -10078,28 +11151,32 @@
       <c r="Q16" s="2">
         <v>23.9</v>
       </c>
+      <c r="R16">
+        <f t="shared" si="4"/>
+        <v>-2.2164073967529934</v>
+      </c>
       <c r="S16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1.2</v>
       </c>
       <c r="T16">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>23.9</v>
       </c>
       <c r="V16">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>7.9181246047624818E-2</v>
       </c>
       <c r="W16">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.3783979009481377</v>
       </c>
       <c r="X16">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.18232155679395459</v>
       </c>
       <c r="Y16">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>3.1738784589374651</v>
       </c>
       <c r="Z16">
@@ -10111,11 +11188,11 @@
         <v>0.18232155679395459</v>
       </c>
       <c r="AB16">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-1.5005835075220182</v>
       </c>
       <c r="AC16">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3.3731407838796299</v>
       </c>
     </row>
@@ -10158,28 +11235,32 @@
       <c r="Q17" s="2">
         <v>29.22</v>
       </c>
+      <c r="R17">
+        <f t="shared" si="4"/>
+        <v>-2.8824035882469876</v>
+      </c>
       <c r="S17">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1</v>
       </c>
       <c r="T17">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>29.22</v>
       </c>
       <c r="V17">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="W17">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.4656802115982779</v>
       </c>
       <c r="X17">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="Y17">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>3.3748534063225533</v>
       </c>
       <c r="Z17">
@@ -10191,11 +11272,11 @@
         <v>0</v>
       </c>
       <c r="AB17">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-1.8971199848858813</v>
       </c>
       <c r="AC17">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3.5319332036512097</v>
       </c>
     </row>
@@ -10238,28 +11319,32 @@
       <c r="Q18" s="2">
         <v>31.63</v>
       </c>
+      <c r="R18">
+        <f t="shared" si="4"/>
+        <v>-2.4079456086518722</v>
+      </c>
       <c r="S18">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.6</v>
       </c>
       <c r="T18">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>31.63</v>
       </c>
       <c r="V18">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>-0.22184874961635639</v>
       </c>
       <c r="W18">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.5000991919157229</v>
       </c>
       <c r="X18">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>-0.51082562376599072</v>
       </c>
       <c r="Y18">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>3.4541060373175574</v>
       </c>
       <c r="Z18">
@@ -10271,12 +11356,41 @@
         <v>-0.51082562376599072</v>
       </c>
       <c r="AB18">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>-1.8018098050815563</v>
       </c>
       <c r="AC18">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3.6189933266497696</v>
+      </c>
+    </row>
+    <row r="50" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA50" s="13">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="51" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA51">
+        <f>LN(AA50)</f>
+        <v>6.9077552789821368</v>
+      </c>
+    </row>
+    <row r="52" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA52">
+        <f>AA51*-0.238</f>
+        <v>-1.6440457563977484</v>
+      </c>
+    </row>
+    <row r="53" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA53">
+        <f>EXP(AA52)</f>
+        <v>0.19319683170169244</v>
+      </c>
+    </row>
+    <row r="54" spans="27:27" x14ac:dyDescent="0.3">
+      <c r="AA54">
+        <f>AA53*0.0673</f>
+        <v>1.30021467735239E-2</v>
       </c>
     </row>
   </sheetData>
@@ -10295,23 +11409,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="c2fb78ee-7f80-47d5-98b2-7e891369b7bb" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B3BEC45979C5C049A19F02E744A428FF" ma:contentTypeVersion="14" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="f5996e32557378a90493e5f03249e0f6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="c2fb78ee-7f80-47d5-98b2-7e891369b7bb" xmlns:ns4="8e80448a-be4d-46ae-83bb-e2adae7741fa" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0d0d7db69a812adcd006be6af9aa5ff0" ns3:_="" ns4:_="">
     <xsd:import namespace="c2fb78ee-7f80-47d5-98b2-7e891369b7bb"/>
@@ -10540,10 +11637,38 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="c2fb78ee-7f80-47d5-98b2-7e891369b7bb" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{546FAC25-7A53-4BE4-87D4-6463C2D97D48}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{212E6E55-4940-49C5-A955-F25080F8975C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c2fb78ee-7f80-47d5-98b2-7e891369b7bb"/>
+    <ds:schemaRef ds:uri="8e80448a-be4d-46ae-83bb-e2adae7741fa"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10566,20 +11691,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{212E6E55-4940-49C5-A955-F25080F8975C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{546FAC25-7A53-4BE4-87D4-6463C2D97D48}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c2fb78ee-7f80-47d5-98b2-7e891369b7bb"/>
-    <ds:schemaRef ds:uri="8e80448a-be4d-46ae-83bb-e2adae7741fa"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
//swatre en van genuchten
</commit_message>
<xml_diff>
--- a/auxfiles/GSSHApedotransfer.xlsx
+++ b/auxfiles/GSSHApedotransfer.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\prgc\lisemgit\openlisem\auxfiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C7D2AE3-4898-488E-8508-8EEE25982C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F24EC14-3F97-4F86-820F-D4E664ECD93C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" activeTab="1" xr2:uid="{EE7E3014-B43F-4E75-BCA9-657834F4F7BD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{EE7E3014-B43F-4E75-BCA9-657834F4F7BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="71">
   <si>
     <t>Sand</t>
   </si>
@@ -344,6 +345,60 @@
   <si>
     <t>pF</t>
   </si>
+  <si>
+    <t>van genuchten</t>
+  </si>
+  <si>
+    <t>alpha</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>Ks</t>
+  </si>
+  <si>
+    <t>cm/min</t>
+  </si>
+  <si>
+    <t>SiC</t>
+  </si>
+  <si>
+    <t>SiCL</t>
+  </si>
+  <si>
+    <t>SC</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>CL</t>
+  </si>
+  <si>
+    <t>Si</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>SiL</t>
+  </si>
+  <si>
+    <t>SCL</t>
+  </si>
+  <si>
+    <t>SL</t>
+  </si>
+  <si>
+    <t>LS</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>Silt</t>
+  </si>
 </sst>
 </file>
 
@@ -491,7 +546,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -521,6 +576,9 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -605,7 +663,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="nl-NL"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -685,7 +743,7 @@
                       <a:cs typeface="+mn-cs"/>
                     </a:defRPr>
                   </a:pPr>
-                  <a:endParaRPr lang="nl-NL"/>
+                  <a:endParaRPr lang="en-US"/>
                 </a:p>
               </c:txPr>
             </c:trendlineLbl>
@@ -847,7 +905,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="918899471"/>
@@ -909,7 +967,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="918901871"/>
@@ -957,7 +1015,877 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="nl-NL"/>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB"/>
+              <a:t>alpha=f(ks)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="log"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.27611351706036746"/>
+                  <c:y val="0.14440653251676874"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="1100" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet3!$S$6:$S$17</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>235.6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>59.800000000000004</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>21.8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>13.200000000000001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.8000000000000007</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.52</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet3!$U$6:$U$17</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>0.14499999999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.124</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>7.4999999999999997E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.5999999999999997E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.02</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.8999999999999997E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.9E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.01</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.7E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>5.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>8.0000000000000002E-3</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.6E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-1CD0-444C-BE84-28434B356488}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1103212928"/>
+        <c:axId val="1103225408"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1103212928"/>
+        <c:scaling>
+          <c:logBase val="10"/>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1103225408"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1103225408"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1103212928"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB"/>
+              <a:t>n=f(Ks)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="log"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.19737751531058617"/>
+                  <c:y val="-4.1666666666666669E-4"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="en-US"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet3!$S$6:$S$17</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>235.6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>59.800000000000004</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>21.8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>13.200000000000001</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.8000000000000007</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.6</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2.52</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet3!$V$6:$V$17</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>2.68</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.2799999999999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.89</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.56</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.41</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.48</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.31</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.23</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.23</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.0900000000000001</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.0900000000000001</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.37</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-B260-49C3-9B8B-4E5EC1AB561A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1103227808"/>
+        <c:axId val="1103228768"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1103227808"/>
+        <c:scaling>
+          <c:logBase val="10"/>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1103228768"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1103228768"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1103227808"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -1037,7 +1965,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="nl-NL"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1127,7 +2055,7 @@
                       <a:cs typeface="+mn-cs"/>
                     </a:defRPr>
                   </a:pPr>
-                  <a:endParaRPr lang="nl-NL"/>
+                  <a:endParaRPr lang="en-US"/>
                 </a:p>
               </c:txPr>
             </c:trendlineLbl>
@@ -1306,7 +2234,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="nl-NL"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1344,7 +2272,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="349205312"/>
@@ -1432,7 +2360,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="nl-NL"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1470,7 +2398,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="349202912"/>
@@ -1518,7 +2446,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="nl-NL"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -1602,7 +2530,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="nl-NL"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1682,7 +2610,7 @@
                       <a:cs typeface="+mn-cs"/>
                     </a:defRPr>
                   </a:pPr>
-                  <a:endParaRPr lang="nl-NL"/>
+                  <a:endParaRPr lang="en-US"/>
                 </a:p>
               </c:txPr>
             </c:trendlineLbl>
@@ -1844,7 +2772,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="348374448"/>
@@ -1906,7 +2834,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="348376368"/>
@@ -1954,7 +2882,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="nl-NL"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -2038,7 +2966,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="nl-NL"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -2118,7 +3046,7 @@
                       <a:cs typeface="+mn-cs"/>
                     </a:defRPr>
                   </a:pPr>
-                  <a:endParaRPr lang="nl-NL"/>
+                  <a:endParaRPr lang="en-US"/>
                 </a:p>
               </c:txPr>
             </c:trendlineLbl>
@@ -2280,7 +3208,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="564138272"/>
@@ -2342,7 +3270,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="564140672"/>
@@ -2390,7 +3318,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="nl-NL"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -2466,7 +3394,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="nl-NL"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -2556,7 +3484,7 @@
                       <a:cs typeface="+mn-cs"/>
                     </a:defRPr>
                   </a:pPr>
-                  <a:endParaRPr lang="nl-NL"/>
+                  <a:endParaRPr lang="en-US"/>
                 </a:p>
               </c:txPr>
             </c:trendlineLbl>
@@ -2718,7 +3646,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="556251872"/>
@@ -2780,7 +3708,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="1564086688"/>
@@ -2828,7 +3756,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="nl-NL"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -2879,7 +3807,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="nl-NL"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -3071,7 +3999,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="2130070832"/>
@@ -3133,7 +4061,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="2130082832"/>
@@ -3181,7 +4109,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="nl-NL"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -3257,7 +4185,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="nl-NL"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -3337,7 +4265,7 @@
                       <a:cs typeface="+mn-cs"/>
                     </a:defRPr>
                   </a:pPr>
-                  <a:endParaRPr lang="nl-NL"/>
+                  <a:endParaRPr lang="en-US"/>
                 </a:p>
               </c:txPr>
             </c:trendlineLbl>
@@ -3499,7 +4427,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="1774120512"/>
@@ -3561,7 +4489,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="1774120032"/>
@@ -3609,7 +4537,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="nl-NL"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -3685,7 +4613,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="nl-NL"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -3759,7 +4687,7 @@
                       <a:cs typeface="+mn-cs"/>
                     </a:defRPr>
                   </a:pPr>
-                  <a:endParaRPr lang="nl-NL"/>
+                  <a:endParaRPr lang="en-US"/>
                 </a:p>
               </c:txPr>
             </c:trendlineLbl>
@@ -3803,7 +4731,7 @@
                       <a:cs typeface="+mn-cs"/>
                     </a:defRPr>
                   </a:pPr>
-                  <a:endParaRPr lang="nl-NL"/>
+                  <a:endParaRPr lang="en-US"/>
                 </a:p>
               </c:txPr>
             </c:trendlineLbl>
@@ -3965,7 +4893,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="167440672"/>
@@ -4027,7 +4955,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="167585584"/>
@@ -4075,7 +5003,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="nl-NL"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -4151,7 +5079,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="nl-NL"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -4245,7 +5173,7 @@
                       <a:cs typeface="+mn-cs"/>
                     </a:defRPr>
                   </a:pPr>
-                  <a:endParaRPr lang="nl-NL"/>
+                  <a:endParaRPr lang="en-US"/>
                 </a:p>
               </c:txPr>
             </c:trendlineLbl>
@@ -4407,7 +5335,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="2009216271"/>
@@ -4469,7 +5397,7 @@
                 <a:cs typeface="+mn-cs"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="nl-NL"/>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="2009214831"/>
@@ -4517,7 +5445,7 @@
       <a:pPr>
         <a:defRPr/>
       </a:pPr>
-      <a:endParaRPr lang="nl-NL"/>
+      <a:endParaRPr lang="en-US"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -4529,6 +5457,86 @@
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors11.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -4889,6 +5897,1038 @@
 </file>
 
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style11.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -10114,6 +12154,205 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>200025</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F9AF0E3-B664-4676-A09A-A422FDE17C61}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="561975" y="1733550"/>
+          <a:ext cx="4514850" cy="3514725"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>147637</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>1390650</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>33337</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{34F41F72-D9D4-3AD9-1F3B-7A2DD227515D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>1376362</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>23812</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>566737</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>100012</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0ABAA864-B541-61DC-EDCD-6F1681F5546A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>219075</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>152176</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDAE594E-89CA-B582-D8F1-879427A2BBBB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="609600" y="6096000"/>
+          <a:ext cx="5705475" cy="2819176"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -10412,26 +12651,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AC7A993-96B8-4AA6-8EF4-C236C394CA84}">
   <dimension ref="F1:AC54"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="8" max="8" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.140625" customWidth="1"/>
+    <col min="8" max="8" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="6:29" x14ac:dyDescent="0.3">
+    <row r="1" spans="6:29" x14ac:dyDescent="0.25">
       <c r="F1" s="4" t="s">
         <v>34</v>
       </c>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
     </row>
-    <row r="3" spans="6:29" x14ac:dyDescent="0.3">
+    <row r="3" spans="6:29" x14ac:dyDescent="0.25">
       <c r="F3" s="5" t="s">
         <v>41</v>
       </c>
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
     </row>
-    <row r="4" spans="6:29" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="6:29" ht="165" x14ac:dyDescent="0.25">
       <c r="F4" s="13" t="s">
         <v>11</v>
       </c>
@@ -10467,7 +12707,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="6:29" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="6:29" ht="18" x14ac:dyDescent="0.25">
       <c r="F5" s="13"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
@@ -10499,7 +12739,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="6:29" ht="45" x14ac:dyDescent="0.3">
+    <row r="6" spans="6:29" ht="47.25" x14ac:dyDescent="0.25">
       <c r="F6" s="13"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
@@ -10565,7 +12805,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="6:29" x14ac:dyDescent="0.3">
+    <row r="7" spans="6:29" x14ac:dyDescent="0.25">
       <c r="G7" s="6" t="s">
         <v>43</v>
       </c>
@@ -10579,7 +12819,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="6:29" x14ac:dyDescent="0.3">
+    <row r="8" spans="6:29" x14ac:dyDescent="0.25">
       <c r="F8" s="1" t="s">
         <v>0</v>
       </c>
@@ -10663,7 +12903,7 @@
         <v>1.9823798288367047</v>
       </c>
     </row>
-    <row r="9" spans="6:29" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="6:29" x14ac:dyDescent="0.25">
       <c r="F9" s="1" t="s">
         <v>1</v>
       </c>
@@ -10747,7 +12987,7 @@
         <v>2.1621729392773008</v>
       </c>
     </row>
-    <row r="10" spans="6:29" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="6:29" x14ac:dyDescent="0.25">
       <c r="F10" s="1" t="s">
         <v>2</v>
       </c>
@@ -10831,7 +13071,7 @@
         <v>2.6851226964585053</v>
       </c>
     </row>
-    <row r="11" spans="6:29" x14ac:dyDescent="0.3">
+    <row r="11" spans="6:29" x14ac:dyDescent="0.25">
       <c r="F11" s="1" t="s">
         <v>3</v>
       </c>
@@ -10915,7 +13155,7 @@
         <v>2.411439497906128</v>
       </c>
     </row>
-    <row r="12" spans="6:29" x14ac:dyDescent="0.3">
+    <row r="12" spans="6:29" x14ac:dyDescent="0.25">
       <c r="F12" s="1" t="s">
         <v>4</v>
       </c>
@@ -10999,7 +13239,7 @@
         <v>3.0344721018699214</v>
       </c>
     </row>
-    <row r="13" spans="6:29" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="6:29" x14ac:dyDescent="0.25">
       <c r="F13" s="1" t="s">
         <v>5</v>
       </c>
@@ -11083,7 +13323,7 @@
         <v>3.3350575791576103</v>
       </c>
     </row>
-    <row r="14" spans="6:29" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="6:29" x14ac:dyDescent="0.25">
       <c r="F14" s="1" t="s">
         <v>6</v>
       </c>
@@ -11167,7 +13407,7 @@
         <v>3.2538567937634464</v>
       </c>
     </row>
-    <row r="15" spans="6:29" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="6:29" x14ac:dyDescent="0.25">
       <c r="F15" s="1" t="s">
         <v>7</v>
       </c>
@@ -11251,7 +13491,7 @@
         <v>3.4830845411343394</v>
       </c>
     </row>
-    <row r="16" spans="6:29" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="6:29" x14ac:dyDescent="0.25">
       <c r="F16" s="1" t="s">
         <v>8</v>
       </c>
@@ -11335,7 +13575,7 @@
         <v>3.3731407838796299</v>
       </c>
     </row>
-    <row r="17" spans="6:29" x14ac:dyDescent="0.3">
+    <row r="17" spans="6:29" x14ac:dyDescent="0.25">
       <c r="F17" s="1" t="s">
         <v>9</v>
       </c>
@@ -11419,7 +13659,7 @@
         <v>3.5319332036512097</v>
       </c>
     </row>
-    <row r="18" spans="6:29" x14ac:dyDescent="0.3">
+    <row r="18" spans="6:29" x14ac:dyDescent="0.25">
       <c r="F18" s="1" t="s">
         <v>10</v>
       </c>
@@ -11503,30 +13743,30 @@
         <v>3.6189933266497696</v>
       </c>
     </row>
-    <row r="50" spans="27:27" x14ac:dyDescent="0.3">
+    <row r="50" spans="27:27" x14ac:dyDescent="0.25">
       <c r="AA50" s="12">
         <v>1000</v>
       </c>
     </row>
-    <row r="51" spans="27:27" x14ac:dyDescent="0.3">
+    <row r="51" spans="27:27" x14ac:dyDescent="0.25">
       <c r="AA51">
         <f>LN(AA50)</f>
         <v>6.9077552789821368</v>
       </c>
     </row>
-    <row r="52" spans="27:27" x14ac:dyDescent="0.3">
+    <row r="52" spans="27:27" x14ac:dyDescent="0.25">
       <c r="AA52">
         <f>AA51*-0.238</f>
         <v>-1.6440457563977484</v>
       </c>
     </row>
-    <row r="53" spans="27:27" x14ac:dyDescent="0.3">
+    <row r="53" spans="27:27" x14ac:dyDescent="0.25">
       <c r="AA53">
         <f>EXP(AA52)</f>
         <v>0.19319683170169244</v>
       </c>
     </row>
-    <row r="54" spans="27:27" x14ac:dyDescent="0.3">
+    <row r="54" spans="27:27" x14ac:dyDescent="0.25">
       <c r="AA54">
         <f>AA53*0.0673</f>
         <v>1.30021467735239E-2</v>
@@ -11550,20 +13790,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF0E24C5-C479-47D4-9617-6832BA07E0D5}">
   <dimension ref="A1:X32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.5546875" customWidth="1"/>
+    <col min="1" max="1" width="21.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
     </row>
-    <row r="6" spans="1:24" ht="79.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:24" ht="79.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>42</v>
       </c>
@@ -11596,7 +13836,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:24" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:24" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2" t="s">
@@ -11627,7 +13867,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:24" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:24" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
@@ -11692,7 +13932,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="6" t="s">
         <v>43</v>
       </c>
@@ -11706,7 +13946,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
@@ -11790,7 +14030,7 @@
         <v>1.9823798288367047</v>
       </c>
     </row>
-    <row r="11" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -11874,7 +14114,7 @@
         <v>2.1621729392773008</v>
       </c>
     </row>
-    <row r="12" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>2</v>
       </c>
@@ -11958,7 +14198,7 @@
         <v>2.6851226964585053</v>
       </c>
     </row>
-    <row r="13" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>3</v>
       </c>
@@ -12042,7 +14282,7 @@
         <v>2.411439497906128</v>
       </c>
     </row>
-    <row r="14" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>4</v>
       </c>
@@ -12126,7 +14366,7 @@
         <v>3.0344721018699214</v>
       </c>
     </row>
-    <row r="15" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>5</v>
       </c>
@@ -12210,7 +14450,7 @@
         <v>3.3350575791576103</v>
       </c>
     </row>
-    <row r="16" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>6</v>
       </c>
@@ -12294,7 +14534,7 @@
         <v>3.2538567937634464</v>
       </c>
     </row>
-    <row r="17" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>7</v>
       </c>
@@ -12378,7 +14618,7 @@
         <v>3.4830845411343394</v>
       </c>
     </row>
-    <row r="18" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>8</v>
       </c>
@@ -12462,7 +14702,7 @@
         <v>3.3731407838796299</v>
       </c>
     </row>
-    <row r="19" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>9</v>
       </c>
@@ -12546,7 +14786,7 @@
         <v>3.5319332036512097</v>
       </c>
     </row>
-    <row r="20" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>10</v>
       </c>
@@ -12630,9 +14870,9 @@
         <v>3.6189933266497696</v>
       </c>
     </row>
-    <row r="21" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="22" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
       <c r="F23" t="s">
         <v>50</v>
       </c>
@@ -12643,7 +14883,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
       <c r="E24">
         <v>0.1</v>
       </c>
@@ -12664,13 +14904,13 @@
         <v>3.3990577914452955</v>
       </c>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
       <c r="E25">
         <f>E24+0.05</f>
         <v>0.15000000000000002</v>
       </c>
       <c r="F25">
-        <f t="shared" ref="F25:F33" si="11">(E25-$H$12)/($D$12-$H$12)</f>
+        <f t="shared" ref="F25:F32" si="11">(E25-$H$12)/($D$12-$H$12)</f>
         <v>0.2645631067961165</v>
       </c>
       <c r="G25">
@@ -12678,15 +14918,15 @@
         <v>2.966877995767073E-2</v>
       </c>
       <c r="H25">
-        <f t="shared" ref="H25:H33" si="13">$I$12/G25</f>
+        <f t="shared" ref="H25:H32" si="13">$I$12/G25</f>
         <v>494.12210481576352</v>
       </c>
       <c r="I25">
-        <f t="shared" ref="I25:I33" si="14">LOG(H25)</f>
+        <f t="shared" ref="I25:I32" si="14">LOG(H25)</f>
         <v>2.6938342827191595</v>
       </c>
     </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.25">
       <c r="E26">
         <f t="shared" ref="E26:E31" si="15">E25+0.05</f>
         <v>0.2</v>
@@ -12708,7 +14948,7 @@
         <v>2.260049556846599</v>
       </c>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:24" x14ac:dyDescent="0.25">
       <c r="E27">
         <f t="shared" si="15"/>
         <v>0.25</v>
@@ -12730,7 +14970,7 @@
         <v>1.9458983351783385</v>
       </c>
     </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.25">
       <c r="E28">
         <f t="shared" si="15"/>
         <v>0.3</v>
@@ -12752,7 +14992,7 @@
         <v>1.6994605627704076</v>
       </c>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.25">
       <c r="E29">
         <f t="shared" si="15"/>
         <v>0.35</v>
@@ -12774,7 +15014,7 @@
         <v>1.4966597285281251</v>
       </c>
     </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:24" x14ac:dyDescent="0.25">
       <c r="E30">
         <f t="shared" si="15"/>
         <v>0.39999999999999997</v>
@@ -12796,7 +15036,7 @@
         <v>1.3243423498152032</v>
       </c>
     </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.25">
       <c r="E31">
         <f t="shared" si="15"/>
         <v>0.44999999999999996</v>
@@ -12818,7 +15058,7 @@
         <v>1.1745305523839262</v>
       </c>
     </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:24" x14ac:dyDescent="0.25">
       <c r="E32">
         <f>E31+0.05</f>
         <v>0.49999999999999994</v>
@@ -12850,7 +15090,599 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D5D5A8B-90A0-4411-8675-844E7B6A353A}">
+  <dimension ref="B3:V17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="18" max="18" width="44.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="K4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="K5" t="s">
+        <v>57</v>
+      </c>
+      <c r="L5" t="s">
+        <v>36</v>
+      </c>
+      <c r="M5" t="s">
+        <v>44</v>
+      </c>
+      <c r="N5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O5" t="s">
+        <v>55</v>
+      </c>
+      <c r="S5" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="T5" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="U5" t="s">
+        <v>54</v>
+      </c>
+      <c r="V5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6" t="s">
+        <v>69</v>
+      </c>
+      <c r="K6">
+        <v>0.495</v>
+      </c>
+      <c r="L6">
+        <f>K6*600</f>
+        <v>297</v>
+      </c>
+      <c r="M6">
+        <f>LN(L6)</f>
+        <v>5.6937321388026998</v>
+      </c>
+      <c r="N6">
+        <v>0.14499999999999999</v>
+      </c>
+      <c r="O6">
+        <v>2.68</v>
+      </c>
+      <c r="Q6">
+        <v>1</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="S6" s="8">
+        <v>235.6</v>
+      </c>
+      <c r="T6" s="10">
+        <f>LN(S6)</f>
+        <v>5.4621354517774314</v>
+      </c>
+      <c r="U6">
+        <v>0.14499999999999999</v>
+      </c>
+      <c r="V6">
+        <v>2.68</v>
+      </c>
+    </row>
+    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="J7" t="s">
+        <v>68</v>
+      </c>
+      <c r="K7">
+        <v>0.2432</v>
+      </c>
+      <c r="L7">
+        <f>K7*600</f>
+        <v>145.91999999999999</v>
+      </c>
+      <c r="M7">
+        <f>LN(L7)</f>
+        <v>4.9830585263260208</v>
+      </c>
+      <c r="N7">
+        <v>0.124</v>
+      </c>
+      <c r="O7">
+        <v>2.2799999999999998</v>
+      </c>
+      <c r="Q7">
+        <v>2</v>
+      </c>
+      <c r="R7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="S7" s="8">
+        <v>59.800000000000004</v>
+      </c>
+      <c r="T7" s="10">
+        <f t="shared" ref="T7:T17" si="0">LN(S7)</f>
+        <v>4.0910056609565864</v>
+      </c>
+      <c r="U7">
+        <v>0.124</v>
+      </c>
+      <c r="V7">
+        <v>2.2799999999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="I8">
+        <v>3</v>
+      </c>
+      <c r="J8" t="s">
+        <v>67</v>
+      </c>
+      <c r="K8">
+        <v>7.3700000000000002E-2</v>
+      </c>
+      <c r="L8">
+        <f>K8*600</f>
+        <v>44.22</v>
+      </c>
+      <c r="M8">
+        <f>LN(L8)</f>
+        <v>3.7891771754293</v>
+      </c>
+      <c r="N8">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="O8">
+        <v>1.89</v>
+      </c>
+      <c r="Q8">
+        <v>3</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="S8" s="8">
+        <v>21.8</v>
+      </c>
+      <c r="T8" s="10">
+        <f t="shared" si="0"/>
+        <v>3.0819099697950434</v>
+      </c>
+      <c r="U8">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="V8">
+        <v>1.89</v>
+      </c>
+    </row>
+    <row r="9" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="I9">
+        <v>4</v>
+      </c>
+      <c r="J9" t="s">
+        <v>64</v>
+      </c>
+      <c r="K9">
+        <v>1.7299999999999999E-2</v>
+      </c>
+      <c r="L9">
+        <f>K9*600</f>
+        <v>10.379999999999999</v>
+      </c>
+      <c r="M9">
+        <f>LN(L9)</f>
+        <v>2.3398808777377424</v>
+      </c>
+      <c r="N9">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="O9">
+        <v>1.56</v>
+      </c>
+      <c r="Q9">
+        <v>4</v>
+      </c>
+      <c r="R9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="S9" s="8">
+        <v>13.200000000000001</v>
+      </c>
+      <c r="T9" s="10">
+        <f t="shared" si="0"/>
+        <v>2.5802168295923251</v>
+      </c>
+      <c r="U9">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="V9">
+        <v>1.56</v>
+      </c>
+    </row>
+    <row r="10" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="I10">
+        <v>5</v>
+      </c>
+      <c r="J10" t="s">
+        <v>65</v>
+      </c>
+      <c r="K10">
+        <v>7.4999999999999997E-3</v>
+      </c>
+      <c r="L10">
+        <f>K10*600</f>
+        <v>4.5</v>
+      </c>
+      <c r="M10">
+        <f>LN(L10)</f>
+        <v>1.5040773967762742</v>
+      </c>
+      <c r="N10">
+        <v>0.02</v>
+      </c>
+      <c r="O10">
+        <v>1.41</v>
+      </c>
+      <c r="Q10">
+        <v>5</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="S10" s="8">
+        <v>6.8000000000000007</v>
+      </c>
+      <c r="T10" s="10">
+        <f t="shared" si="0"/>
+        <v>1.9169226121820611</v>
+      </c>
+      <c r="U10">
+        <v>0.02</v>
+      </c>
+      <c r="V10">
+        <v>1.41</v>
+      </c>
+    </row>
+    <row r="11" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="I11">
+        <v>6</v>
+      </c>
+      <c r="J11" t="s">
+        <v>66</v>
+      </c>
+      <c r="K11">
+        <v>2.18E-2</v>
+      </c>
+      <c r="L11">
+        <f>K11*600</f>
+        <v>13.08</v>
+      </c>
+      <c r="M11">
+        <f>LN(L11)</f>
+        <v>2.5710843460290524</v>
+      </c>
+      <c r="N11">
+        <v>5.8999999999999997E-2</v>
+      </c>
+      <c r="O11">
+        <v>1.48</v>
+      </c>
+      <c r="Q11">
+        <v>6</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="S11" s="8">
+        <v>3</v>
+      </c>
+      <c r="T11" s="10">
+        <f t="shared" si="0"/>
+        <v>1.0986122886681098</v>
+      </c>
+      <c r="U11">
+        <v>5.8999999999999997E-2</v>
+      </c>
+      <c r="V11">
+        <v>1.48</v>
+      </c>
+    </row>
+    <row r="12" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="I12">
+        <v>7</v>
+      </c>
+      <c r="J12" t="s">
+        <v>62</v>
+      </c>
+      <c r="K12">
+        <v>4.3E-3</v>
+      </c>
+      <c r="L12">
+        <f>K12*600</f>
+        <v>2.58</v>
+      </c>
+      <c r="M12">
+        <f>LN(L12)</f>
+        <v>0.94778939893352609</v>
+      </c>
+      <c r="N12">
+        <v>1.9E-2</v>
+      </c>
+      <c r="O12">
+        <v>1.31</v>
+      </c>
+      <c r="Q12">
+        <v>7</v>
+      </c>
+      <c r="R12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="S12" s="8">
+        <v>2</v>
+      </c>
+      <c r="T12" s="10">
+        <f t="shared" si="0"/>
+        <v>0.69314718055994529</v>
+      </c>
+      <c r="U12">
+        <v>1.9E-2</v>
+      </c>
+      <c r="V12">
+        <v>1.31</v>
+      </c>
+    </row>
+    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="I13">
+        <v>8</v>
+      </c>
+      <c r="J13" t="s">
+        <v>59</v>
+      </c>
+      <c r="K13">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="L13">
+        <f>K13*600</f>
+        <v>0.72</v>
+      </c>
+      <c r="M13">
+        <f>LN(L13)</f>
+        <v>-0.3285040669720361</v>
+      </c>
+      <c r="N13">
+        <v>0.01</v>
+      </c>
+      <c r="O13">
+        <v>1.23</v>
+      </c>
+      <c r="Q13">
+        <v>8</v>
+      </c>
+      <c r="R13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="S13" s="8">
+        <v>2</v>
+      </c>
+      <c r="T13" s="10">
+        <f t="shared" si="0"/>
+        <v>0.69314718055994529</v>
+      </c>
+      <c r="U13">
+        <v>0.01</v>
+      </c>
+      <c r="V13">
+        <v>1.23</v>
+      </c>
+    </row>
+    <row r="14" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="I14">
+        <v>9</v>
+      </c>
+      <c r="J14" t="s">
+        <v>60</v>
+      </c>
+      <c r="K14">
+        <v>2E-3</v>
+      </c>
+      <c r="L14">
+        <f>K14*600</f>
+        <v>1.2</v>
+      </c>
+      <c r="M14">
+        <f>LN(L14)</f>
+        <v>0.18232155679395459</v>
+      </c>
+      <c r="N14">
+        <v>2.7E-2</v>
+      </c>
+      <c r="O14">
+        <v>1.23</v>
+      </c>
+      <c r="Q14">
+        <v>9</v>
+      </c>
+      <c r="R14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="S14" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="T14" s="10">
+        <f t="shared" si="0"/>
+        <v>0.18232155679395459</v>
+      </c>
+      <c r="U14">
+        <v>2.7E-2</v>
+      </c>
+      <c r="V14">
+        <v>1.23</v>
+      </c>
+    </row>
+    <row r="15" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="I15">
+        <v>10</v>
+      </c>
+      <c r="J15" t="s">
+        <v>58</v>
+      </c>
+      <c r="K15">
+        <v>2.9999999999999997E-4</v>
+      </c>
+      <c r="L15">
+        <f>K15*600</f>
+        <v>0.18</v>
+      </c>
+      <c r="M15">
+        <f>LN(L15)</f>
+        <v>-1.7147984280919266</v>
+      </c>
+      <c r="N15">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="O15">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="Q15">
+        <v>10</v>
+      </c>
+      <c r="R15" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="S15" s="8">
+        <v>1</v>
+      </c>
+      <c r="T15" s="10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="U15">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="V15">
+        <v>1.0900000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="I16">
+        <v>11</v>
+      </c>
+      <c r="J16" t="s">
+        <v>61</v>
+      </c>
+      <c r="K16">
+        <v>3.3E-3</v>
+      </c>
+      <c r="L16">
+        <f>K16*600</f>
+        <v>1.98</v>
+      </c>
+      <c r="M16">
+        <f>LN(L16)</f>
+        <v>0.68309684470644383</v>
+      </c>
+      <c r="N16">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="O16">
+        <v>1.0900000000000001</v>
+      </c>
+      <c r="Q16">
+        <v>11</v>
+      </c>
+      <c r="R16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="S16" s="9">
+        <v>0.6</v>
+      </c>
+      <c r="T16" s="10">
+        <f t="shared" si="0"/>
+        <v>-0.51082562376599072</v>
+      </c>
+      <c r="U16">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="V16">
+        <v>1.0900000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="9:22" x14ac:dyDescent="0.25">
+      <c r="I17">
+        <v>12</v>
+      </c>
+      <c r="J17" t="s">
+        <v>63</v>
+      </c>
+      <c r="K17">
+        <v>4.1999999999999997E-3</v>
+      </c>
+      <c r="L17">
+        <f>K17*600</f>
+        <v>2.52</v>
+      </c>
+      <c r="M17">
+        <f>LN(L17)</f>
+        <v>0.9242589015233319</v>
+      </c>
+      <c r="N17">
+        <v>1.6E-2</v>
+      </c>
+      <c r="O17">
+        <v>1.37</v>
+      </c>
+      <c r="Q17">
+        <v>12</v>
+      </c>
+      <c r="R17" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="S17" s="14">
+        <v>2.52</v>
+      </c>
+      <c r="T17" s="10">
+        <f t="shared" si="0"/>
+        <v>0.9242589015233319</v>
+      </c>
+      <c r="U17">
+        <v>1.6E-2</v>
+      </c>
+      <c r="V17">
+        <v>1.37</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="I6:O17">
+    <sortCondition ref="I6:I17"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="c2fb78ee-7f80-47d5-98b2-7e891369b7bb" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B3BEC45979C5C049A19F02E744A428FF" ma:contentTypeVersion="14" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="f5996e32557378a90493e5f03249e0f6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="c2fb78ee-7f80-47d5-98b2-7e891369b7bb" xmlns:ns4="8e80448a-be4d-46ae-83bb-e2adae7741fa" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0d0d7db69a812adcd006be6af9aa5ff0" ns3:_="" ns4:_="">
     <xsd:import namespace="c2fb78ee-7f80-47d5-98b2-7e891369b7bb"/>
@@ -13079,14 +15911,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="c2fb78ee-7f80-47d5-98b2-7e891369b7bb" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -13097,6 +15921,23 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F2FDDBA-8E4A-41B0-9357-134C9F5B7B79}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="8e80448a-be4d-46ae-83bb-e2adae7741fa"/>
+    <ds:schemaRef ds:uri="c2fb78ee-7f80-47d5-98b2-7e891369b7bb"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{212E6E55-4940-49C5-A955-F25080F8975C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -13115,23 +15956,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F2FDDBA-8E4A-41B0-9357-134C9F5B7B79}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="8e80448a-be4d-46ae-83bb-e2adae7741fa"/>
-    <ds:schemaRef ds:uri="c2fb78ee-7f80-47d5-98b2-7e891369b7bb"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{546FAC25-7A53-4BE4-87D4-6463C2D97D48}">
   <ds:schemaRefs>

</xml_diff>